<commit_message>
Fill real product specs for Decotica cosmetology models
Add real technical characteristics, technologies and warranty pulled from
product card pages: Solalux Combi (hybrid Alex/Nd:YAG laser), Esther
(fractional IPL/FPL), Pinacle (microneedle RF/MNRF), Curelux (LED photo-
therapy). Correct Pinacle technology to microneedle RF.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012Rw9dvcAKokoAsKsBSt35U
</commit_message>
<xml_diff>
--- a/medford_kosmetologiya_v2.xlsx
+++ b/medford_kosmetologiya_v2.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -755,32 +755,49 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Заполнить вручную</t>
+          <t>Характеристики товаров</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Характеристики товаров, страна, наличие, РУ, цены, кейсы, ФИО автора, телефон</t>
+          <t>Заполнены с карточек товаров medford.ru (технологии, параметры, гарантия)</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Проставлены плейсхолдеры [ ] / «уточнять» — брать с карточек товаров и из данных компании</t>
+          <t>Solalux/Esther/Pinacle/Curelux — реальные ТТХ</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>Заполнить вручную</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Страна производства, наличие, статус РУ Росздравнадзора, цены, кейсы, ФИО автора, телефон</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>На страницах не указаны — плейсхолдеры [ ] / «уточнять»</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
           <t>URL раздела</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>https://medford.ru/catalog/kosmetologiya/</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>SECTION_CODE = kosmetologiya · 4 подкатегории</t>
         </is>
@@ -4070,12 +4087,12 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Лазер (многофункциональная система)</t>
+          <t>Лазер (александрит 755 нм + Nd:YAG 1064 нм)</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>Эпиляция, омоложение, лечение кожи</t>
+          <t>Эпиляция всех фототипов, сосудистые патологии, пигментация, омоложение, стрии, рубцы</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -4111,12 +4128,12 @@
       <c r="S4" s="3" t="inlineStr"/>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>[Заполнить с карточки товара на medford.ru]</t>
+          <t>Гибридная платформа: александрит 755 нм + Nd:YAG 1064 нм в одной манипуле|Технология Hybrid Alex/Nd:YAG — одновременная подача двух длин волн|7 размеров светового пятна без замены насадок (расходники до −40%)|Режимы: Alexandrite 755, Nd:YAG 1064, Hybrid 755/1064; Smart Mode|Задачи: эпиляция, сосудистые, пигментация, омоложение, стрии, рубцы, онихомикоз</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>Многофункциональная лазерная система — комбинированные процедуры</t>
+          <t>Гибридная лазерная система: александрит 755 нм + Nd:YAG 1064 нм</t>
         </is>
       </c>
       <c r="V4" s="3" t="inlineStr">
@@ -4174,12 +4191,12 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>IPL (интенсивный импульсный свет)</t>
+          <t>IPL / FPL (фракционный импульсный свет)</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>Фотоомоложение, лечение акне, пигментации, эпиляция</t>
+          <t>Фотоомоложение, сосудистые, пигментация, акне/постакне, эпиляция (I–III фототип)</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
@@ -4204,7 +4221,7 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>уточнять</t>
+          <t>до 24 месяцев</t>
         </is>
       </c>
       <c r="R5" s="3" t="inlineStr">
@@ -4215,12 +4232,12 @@
       <c r="S5" s="3" t="inlineStr"/>
       <c r="T5" s="3" t="inlineStr">
         <is>
-          <t>[Заполнить с карточки товара на medford.ru]</t>
+          <t>Фракционный IPL/FPL, технология 140 multi-cell|Флюенс 1–32 Дж/см², импульс 0,2–40 мс, пятно 42,6 × 14,3 мм|7 экспертных фильтров: 415/530/560/590/640/690/755 нм|Режимы Stamp и In-motion; встроенные SMART-протоколы|Задачи: сосудистые, пигментация, акне/постакне, термолифтинг, эпиляция</t>
         </is>
       </c>
       <c r="U5" s="3" t="inlineStr">
         <is>
-          <t>IPL-аппарат — фототерапия и фотоомоложение</t>
+          <t>Фракционный IPL/FPL-аппарат для фотоомоложения и коррекции кожи</t>
         </is>
       </c>
       <c r="V5" s="3" t="inlineStr">
@@ -4278,12 +4295,12 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>RF (радиочастотный лифтинг)</t>
+          <t>Микроигольчатый RF (MNRF)</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>Подтяжка кожи, стимуляция коллагена</t>
+          <t>Термолифтинг, ремоделирование кожи, рубцы постакне, морщины, стрии, дряблость</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
@@ -4308,7 +4325,7 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>уточнять</t>
+          <t>24 месяца</t>
         </is>
       </c>
       <c r="R6" s="3" t="inlineStr">
@@ -4319,12 +4336,12 @@
       <c r="S6" s="3" t="inlineStr"/>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>[Заполнить с карточки товара на medford.ru]</t>
+          <t>Микроигольчатый RF (MNRF), частота 1 и 2 МГц, мощность 40 Вт|Технология DOUBLE Shot; встроенные SMART-протоколы|3 типа картриджей: изолир./неизолир. иглы 36 pin, глубина 0,5–4 мм; неинвазивные электроды|Шаг глубины 0,1 мм, ресурс картриджа 3000 проколов; процедура 15–20 мин|Задачи: постакне и рубцы, морщины, стрии, дряблость, локальный гипергидроз</t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
         <is>
-          <t>Аппарат для RF-лифтинга — радиочастотная подтяжка кожи</t>
+          <t>Микроигольчатый RF-аппарат для фракционного термолифтинга и ремоделирования кожи</t>
         </is>
       </c>
       <c r="V6" s="3" t="inlineStr">
@@ -4382,12 +4399,12 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Фототерапия (фотобиомодуляция, PDT)</t>
+          <t>LED-фототерапия (ФБМ + ФДТ)</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>Фотобиомодуляция, фотодинамическая терапия, регенерация</t>
+          <t>Восстановление после процедур, акне/розацеа, заживление ран, anti-age, трихология</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -4423,12 +4440,12 @@
       <c r="S7" s="3" t="inlineStr"/>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>[Заполнить с карточки товара на medford.ru]</t>
+          <t>Светодиодная фототерапия: фотобиомодуляция (ФБМ) + фотодинамическая терапия (ФДТ)|4 длины волны: 415 (синий), 585 (жёлтый), 635 (красный), 830 нм (ИК)|Mix-протокол — до 3 длин волн одновременно; матрица линз OML|SMART-протоколы; процедура 10–50 мин; 0 ₽ на расходники|Задачи: акне/розацеа, трихология, заживление ран, восстановление, anti-age</t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr">
         <is>
-          <t>Фотобиомодуляция и фотодинамическая терапия (PDT)</t>
+          <t>Светодиодная система для фотобиомодуляции и фотодинамической терапии</t>
         </is>
       </c>
       <c r="V7" s="3" t="inlineStr">
@@ -4440,7 +4457,7 @@
     <row r="9">
       <c r="E9" t="inlineStr">
         <is>
-          <t>Все 4 товара — из живого каталога medford.ru на дату страницы. Бренд Decotica, цена «по запросу». Спецификации, страна, наличие и РУ — заполнить с карточек товаров (на странице категории их нет).</t>
+          <t>Все 4 товара — из живого каталога medford.ru. Бренд Decotica, цена «по запросу». Характеристики и гарантия — с карточек товаров. Осталось уточнить только страну производства, наличие и статус РУ Росздравнадзора (на страницах не указаны).</t>
         </is>
       </c>
     </row>
@@ -4617,12 +4634,12 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Лазер (многофункц.)</t>
+          <t>Лазер Alex 755 + Nd:YAG 1064</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>Эпиляция, омоложение, лечение кожи</t>
+          <t>Эпиляция, сосудистые, пигментация, омоложение</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -4637,7 +4654,7 @@
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>от 12 мес</t>
+          <t>уточнять</t>
         </is>
       </c>
       <c r="P4" s="3" t="inlineStr">
@@ -4695,12 +4712,12 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>IPL</t>
+          <t>IPL / FPL (140 multi-cell)</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>Фотоомоложение, акне, пигментация, эпиляция</t>
+          <t>Фотоомоложение, акне, пигментация, сосудистые, эпиляция</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
@@ -4715,7 +4732,7 @@
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>от 12 мес</t>
+          <t>до 24 мес</t>
         </is>
       </c>
       <c r="P5" s="3" t="inlineStr">
@@ -4773,12 +4790,12 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>RF</t>
+          <t>Микроигольчатый RF (MNRF)</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>Подтяжка кожи, стимуляция коллагена</t>
+          <t>Термолифтинг, рубцы постакне, морщины, стрии</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
@@ -4793,7 +4810,7 @@
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>от 12 мес</t>
+          <t>24 мес</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
@@ -4851,12 +4868,12 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Фотобиомодуляция / PDT</t>
+          <t>LED-фототерапия (ФБМ + ФДТ)</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>Регенерация, фотодинамическая терапия</t>
+          <t>Восстановление, акне/розацеа, заживление, anti-age</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -4871,7 +4888,7 @@
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>от 12 мес</t>
+          <t>уточнять</t>
         </is>
       </c>
       <c r="P7" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Set placeholder author name and company phone
Random placeholder author (Марина Ковалёва) in section UF and expert block
for manual replacement; add company phone +7 (499) 495-48-21 to SEO block.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012Rw9dvcAKokoAsKsBSt35U
</commit_message>
<xml_diff>
--- a/medford_kosmetologiya_v2.xlsx
+++ b/medford_kosmetologiya_v2.xlsx
@@ -777,12 +777,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Страна производства, наличие, статус РУ Росздравнадзора, цены, кейсы, ФИО автора, телефон</t>
+          <t>Страна производства, наличие, статус РУ Росздравнадзора, цены, кейсы (08_CASES)</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>На страницах не указаны — плейсхолдеры [ ] / «уточнять»</t>
+          <t>На страницах не указаны — плейсхолдеры [ ] / «уточнять». ФИО автора — рандомный, заменить</t>
         </is>
       </c>
     </row>
@@ -3376,7 +3376,7 @@
       <c r="L4" s="3" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>[ФИО автора]</t>
+          <t>Марина Ковалёва</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
@@ -3386,7 +3386,7 @@
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>Товары — реальный каталог medford.ru (4 модели Decotica); тексты — триплеты SERP</t>
+          <t>ФИО автора — рандомный плейсхолдер, заменить вручную. Товары — реальный каталог medford.ru</t>
         </is>
       </c>
     </row>
@@ -5548,12 +5548,12 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>[ФИО эксперта]</t>
+          <t>Марина Ковалёва</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Специалист по косметологическому оборудованию, Medford · Опыт [N лет]</t>
+          <t>Специалист по косметологическому оборудованию, Medford · Опыт [N лет] · ФИО — рандомный плейсхолдер, заменить</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -6044,7 +6044,7 @@
       <c r="F25" s="3" t="inlineStr"/>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Оплата — по счёту для юридических лиц и ИП. Доставка товаров — по всей России. Гарантия — от 12 месяцев с сервисной поддержкой; предоставляется обучение работе на аппарате. ООО «Медфорд» работает с 2009 года. Телефон для консультаций: [телефон].</t>
+          <t>Оплата — по счёту для юридических лиц и ИП. Доставка товаров — по всей России. Гарантия — от 12 месяцев с сервисной поддержкой; предоставляется обучение работе на аппарате. ООО «Медфорд» работает с 2009 года. Телефон для консультаций: +7 (499) 495-48-21.</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">

</xml_diff>